<commit_message>
test(pivots): rebuild pivot references from a Calibri 11, English-caption seed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KTccUzeFqqMqTthqgFm9H
</commit_message>
<xml_diff>
--- a/tests/fixtures/xlsx-pivots/pivot-collapsed-item.xlsx
+++ b/tests/fixtures/xlsx-pivots/pivot-collapsed-item.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/julianshen/prj/officeview/.worktrees/pivots/tests/fixtures/xlsx-pivots/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ABFFA97D-B5DE-AC44-9BB4-B99FB2E38016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{142B41DC-E3C9-E944-AB35-F8ECFADC6D12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5080" yWindow="1820" windowWidth="28240" windowHeight="17320" xr2:uid="{044873AD-994E-A242-BEC3-CCCD5EADFF8E}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="181029"/>
   <pivotCaches>
-    <pivotCache cacheId="1403" r:id="rId3"/>
+    <pivotCache cacheId="2094" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -81,35 +81,40 @@
     <t>East</t>
   </si>
   <si>
-    <t>列標籤</t>
+    <t>Row Labels</t>
   </si>
   <si>
-    <t>總計</t>
+    <t>Column Labels</t>
   </si>
   <si>
-    <t>欄標籤</t>
+    <t>Grand Total</t>
   </si>
   <si>
-    <t>加總 - Sales</t>
+    <t>Sum of Sales 的加總</t>
   </si>
   <si>
-    <t>加總 - Sales 的加總</t>
+    <t>Sum of Sales</t>
   </si>
   <si>
-    <t>加總 - Units 的加總</t>
+    <t>Sum of Units 的加總</t>
   </si>
   <si>
-    <t>加總 - Units</t>
+    <t>Sum of Units</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <name val="新細明體"/>
       <family val="2"/>
       <charset val="136"/>
@@ -117,10 +122,9 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="新細明體"/>
-      <family val="2"/>
+      <name val="Wawati TC"/>
+      <family val="3"/>
       <charset val="136"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -179,7 +183,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Julian Shen" refreshedDate="46324.251751967589" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="36" xr:uid="{ACFBA65F-A556-CF48-AE79-85CC1FCB028C}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Julian Shen" refreshedDate="46324.27183229167" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="36" xr:uid="{6D0D7B28-7BA4-D845-B57D-7D154BE39B4D}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:E37" sheet="Data"/>
   </cacheSource>
@@ -482,7 +486,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0E335153-2009-4949-B2E0-C4B3FBEEF68D}" name="樞紐分析表1" cacheId="1403" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3FBD5118-D9A9-0C4C-A9C7-023E41C87F08}" name="樞紐分析表2" cacheId="2094" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Grand Total" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Row Labels" colHeaderCaption="Column Labels">
   <location ref="A3:I19" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
@@ -595,8 +599,8 @@
     </i>
   </colItems>
   <dataFields count="2">
-    <dataField name="加總 - Sales" fld="3" baseField="0" baseItem="0"/>
-    <dataField name="加總 - Units" fld="4" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Sales" fld="3" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Units" fld="4" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -926,19 +930,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D125325-681A-2147-8208-660E90EC2272}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FF294D8-3310-B842-B316-957631AAF6FC}">
   <dimension ref="A3:I19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="7" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:9">
       <c r="B3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -952,7 +961,7 @@
         <v>2024</v>
       </c>
       <c r="H4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I4" t="s">
         <v>17</v>
@@ -963,19 +972,19 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
         <v>18</v>
       </c>
       <c r="F5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G5" t="s">
         <v>18</v>
@@ -1320,7 +1329,7 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B19" s="4">
         <v>40972.090000000004</v>
@@ -1348,7 +1357,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>